<commit_message>
Add multilogue L1b validation and VPS deployment support
</commit_message>
<xml_diff>
--- a/outputs/validation-sprint/8_STEM_SpeakerX/phase-v/validation_matrix_speakerx.xlsx
+++ b/outputs/validation-sprint/8_STEM_SpeakerX/phase-v/validation_matrix_speakerx.xlsx
@@ -134,14 +134,14 @@
     <t>generated_at</t>
   </si>
   <si>
-    <t>2026-06-22T03:10:27.360Z</t>
+    <t>2026-07-13T16:07:55.583Z</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -151,17 +151,35 @@
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFF"/>
+      <sz val="10"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <color rgb="203036"/>
+      <sz val="10"/>
+      <name val="Aptos"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="173F4F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="F4F7F7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -169,13 +187,47 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="173F4F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="hair">
+        <color rgb="D9E1E3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -515,246 +567,279 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:Z2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="21" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="17" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12" style="1" customWidth="1"/>
+    <col min="3" max="3" width="35" style="1" customWidth="1"/>
+    <col min="4" max="4" width="38" style="1" customWidth="1"/>
+    <col min="5" max="5" width="34" style="1" customWidth="1"/>
+    <col min="6" max="6" width="38" style="1" customWidth="1"/>
+    <col min="7" max="7" width="30" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23" style="1" customWidth="1"/>
+    <col min="9" max="9" width="27" style="1" customWidth="1"/>
+    <col min="10" max="10" width="35" style="1" customWidth="1"/>
+    <col min="11" max="11" width="38" style="1" customWidth="1"/>
+    <col min="12" max="12" width="34" style="1" customWidth="1"/>
+    <col min="13" max="13" width="38" style="1" customWidth="1"/>
+    <col min="14" max="14" width="30" style="1" customWidth="1"/>
+    <col min="15" max="15" width="23" style="1" customWidth="1"/>
+    <col min="16" max="16" width="27" style="1" customWidth="1"/>
+    <col min="17" max="17" width="28" style="1" customWidth="1"/>
+    <col min="18" max="19" width="30" style="1" customWidth="1"/>
+    <col min="20" max="24" width="25" style="1" customWidth="1"/>
+    <col min="25" max="25" width="18" style="1" customWidth="1"/>
+    <col min="26" max="26" width="19" style="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" ht="21" customHeight="1" spans="1:26" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G2">
+      <c r="C2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="5">
         <v>27.027731</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="5">
         <v>240.99727</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="5">
         <v>0.833045</v>
       </c>
-      <c r="J2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K2" t="s">
-        <v>28</v>
-      </c>
-      <c r="L2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N2">
+      <c r="J2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2" s="5">
         <v>36.106097</v>
       </c>
-      <c r="O2">
+      <c r="O2" s="5">
         <v>272.067066</v>
       </c>
-      <c r="P2">
+      <c r="P2" s="5">
         <v>0.91822</v>
       </c>
-      <c r="Q2" t="s">
-        <v>28</v>
-      </c>
-      <c r="R2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S2" t="s">
-        <v>28</v>
-      </c>
-      <c r="T2" t="s">
-        <v>28</v>
-      </c>
-      <c r="U2" t="s">
-        <v>28</v>
-      </c>
-      <c r="V2" t="s">
-        <v>28</v>
-      </c>
-      <c r="W2" t="s">
-        <v>28</v>
-      </c>
-      <c r="X2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y2" t="s">
+      <c r="Q2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="T2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="U2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="Z2" s="5" t="s">
         <v>30</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <autoFilter ref="A1:Z1"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="21" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="18" style="1" customWidth="1"/>
+    <col min="2" max="2" width="38" style="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" ht="21" customHeight="1" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" ht="21" customHeight="1" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" ht="21" customHeight="1" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" ht="21" customHeight="1" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" ht="21" customHeight="1" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" ht="21" customHeight="1" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" ht="21" customHeight="1" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <autoFilter ref="A1:B1"/>
+  <pageSetup orientation="portrait" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>